<commit_message>
Regenerate Excel export to match round 2 HTML changes
Updates the Excel mirror of notifications-framework.html: renamed
resolve column, single Data Source value, paired retention lists,
and notes for the two still-open clarification items.

https://claude.ai/code/session_0123GvTUP4hUPYgJuh7p63Hm
</commit_message>
<xml_diff>
--- a/notifications-framework.xlsx
+++ b/notifications-framework.xlsx
@@ -455,9 +455,9 @@
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -489,7 +489,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>How User Resolves</t>
+          <t>Where User Can Resolve</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -508,7 +508,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Interactions Report</t>
@@ -536,18 +536,28 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Data Source (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Original data source (primary)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Teams Homepage
+Interactions Report
+Interactions Hub Calendar view</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 month "past due" after date of interaction
+Indefinitely
+1 week past date of notes logged</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
-    <row r="3">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Interactions Report</t>
@@ -575,18 +585,28 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Teams Homepage
+Interactions Report
+Interactions Hub Calendar view</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 month past due after date of interaction
+Indefinitely
+1 week past date of notes logged</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr"/>
     </row>
-    <row r="4">
+    <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Interactions Report</t>
@@ -614,18 +634,28 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Data Source (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Original data source (primary)</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Teams Homepage
+Interactions Report
+Interactions Hub Tasks tab</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 month past due after date of interaction
+Indefinitely
+1 month past due date</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
-    <row r="5">
+    <row r="5" ht="90" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Interactions Report</t>
@@ -653,18 +683,32 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
+          <t>Activity Feed
+Teams Homepage
+Interactions Report
+Interactions Hub Tasks tab</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 month past due after date of interaction
+Indefinitely
+1 month past due date</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>[C4-Row4] Retention inferred from "Upcoming Task" family (Row 3) — not given separately in feedback. Confirm or provide distinct retention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Interactions Report</t>
@@ -692,18 +736,28 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Teams Homepage
+Interactions Report (shows as deleted)
+Interactions Hub Tasks tab</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 month past due after date of interaction
+Indefinitely
+1 week past date of update</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr"/>
     </row>
-    <row r="7">
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Opportunity Details / Opportunities</t>
@@ -716,7 +770,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>After user creates a change to Accountable Banker, Deal State, Est. Close Date, Jnl, Frc, Probability on a deal this user is staffed on</t>
+          <t>Banker updates a key deal attribute, such as (but not limited to) probability, coverage, estimated close date, or estimated fee.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -731,22 +785,30 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Original data source NEW – Changelog (primary)</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>[C2] Trigger text partially legible in source screenshot — verify wording. [C6] 'NEW – Changelog' label meaning not explained in source.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Activity Feed
+Opportunity Details
+Opportunities widget
+Change Log
+Weekly Change Digest</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 week past date of alert/update
+1 week past date of alert/update
+1 year past date of alert/update
+1 month past date of alert/update</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Opportunity Details / Opportunities</t>
@@ -774,18 +836,32 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Data Source (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Original data source (primary)</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Textbot
+Opportunity Details
+Opportunities widget
+Change Log
+Weekly Change Digest</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 month past date of alert/update
+1 week past date of alert/update
+1 week past date of alert/update
+1 year past date of alert/update
+1 month past date of alert/update</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
-    <row r="9">
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Opportunity Details / Opportunities</t>
@@ -813,18 +889,30 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Opportunity Details
+Opportunities widget
+Change Log
+Weekly Change Digest</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 week past date of alert/update
+1 week past date of alert/update
+1 year past date of alert/update
+1 month past date of alert/update</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
-    <row r="10">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Engagement Health</t>
@@ -837,7 +925,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Banking's last interaction date coming past due in 3 days; My last Interaction date coming past due in 5 days</t>
+          <t>Banking's last interaction date is coming due in, or My Last Interaction Date is coming due — both within 2 weeks</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -852,22 +940,26 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Data Source (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Original data source (primary)</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>[C5] Unclear if 3-day and 5-day thresholds are one combined rule or two separate scenarios.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>Activity Feed
+Engagement Health
+Interactions page</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 year "past due" (after which client marked 'inactive')
+Indefinitely (after 1 year past due, client becomes 'inactive')</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Signals</t>
@@ -895,18 +987,24 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Data Source (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Signals</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+90 days</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
-    <row r="12">
+    <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Approvals Queue</t>
@@ -934,18 +1032,28 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
+          <t>Activity Feed
+Opportunity Details</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 week past date of update</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>[C4-Row11] Trigger logic copy not explicitly updated in feedback (only retention given) — left as original.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Approvals Queue</t>
@@ -958,12 +1066,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>When another banker requests a client tier change, for example, that this banker needs to approve</t>
+          <t>Another banker on same deal team requests a deal attribute change that requires approval.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Update</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -973,18 +1081,26 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary), Operations (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>No trail (primary)</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
+          <t>Activity Feed</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Type changed from Alert to Update per feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Hierarchy Cases</t>
@@ -1012,18 +1128,24 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Consolidated data trail (primary)</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>Activity Feed
+Opportunity Details</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update
+1 week past date of update</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
     </row>
-    <row r="15">
+    <row r="15" ht="90" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Hierarchy Cases</t>
@@ -1036,12 +1158,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>When another banker requests a client legal entity change, for example, that this banker has clearance to approve</t>
+          <t>Another banker on same deal team requests a change to the status of a covered account which requires approval.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Update</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1051,18 +1173,22 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Operations (primary)</t>
+          <t>Data Source</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Consolidated data trail (primary)</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>Activity Feed</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>90 days past date of alert/update</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>[C3] Operations appears highlighted as primary resolve path; Activity Feed state is visually ambiguous in source screenshot.</t>
+          <t>Type changed from Alert to Update per feedback.</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1107,21 +1233,28 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>3. 'For How Long' column is currently blank — fill in retention values if known.</t>
+          <t>3. 'Where Data Is Stored' and 'For How Long' are paired line-by-line (line 1 of each column corresponds to line 1 of the other, etc). Keep them in sync if you add/remove a line.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>4. The 'Clarification Flag / Notes' column lists open questions [C1]-[C7] from the original review.</t>
+          <t>4. 'Where User Can Resolve' is now a single value (Data Source) for every row per latest feedback.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>5. Send this file back and changes will be applied to notifications-framework.html.</t>
+          <t>5. The 'Clarification Flag / Notes' column lists open questions still requiring confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>6. Send this file back and changes will be applied to notifications-framework.html.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply round 3 feedback: per-trigger notify/resolve values
Confirms C4-Row4 and C4-Row11 as correct. Replaces the uniform
"Where User Is Notified" and "Where User Can Resolve" values with the
trigger-by-trigger spec provided, including N/A and "Depends" entries.
Regenerates the Excel mirror to match.

https://claude.ai/code/session_0123GvTUP4hUPYgJuh7p63Hm
</commit_message>
<xml_diff>
--- a/notifications-framework.xlsx
+++ b/notifications-framework.xlsx
@@ -531,12 +531,15 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed, Teams, Int. Hub, Int. Report</t>
+          <t>Activity Feed
+Teams Textbot
+Int. Hub</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>Interactions Report
+Teams Textbot</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -580,12 +583,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed, Teams, Int. Hub, Int. Report</t>
+          <t>Activity Feed
+Teams Textbot
+Int. Hub</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -629,12 +634,13 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Int. Hub</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>Interactions Report</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -678,12 +684,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -704,7 +710,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>[C4-Row4] Retention inferred from "Upcoming Task" family (Row 3) — not given separately in feedback. Confirm or provide distinct retention.</t>
+          <t>[C4-Row4] Retention inferred from "Upcoming Task" family (Row 3) — confirmed correct by stakeholder.</t>
         </is>
       </c>
     </row>
@@ -731,12 +737,13 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Int. Hub</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -780,12 +787,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Opportunities Page
+Opportunities Widget</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -831,12 +840,15 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Opportunities Page
+Opportunities Widget</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>Opportunities Widget
+Teams Textbot</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -884,12 +896,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Opportunities Page
+Opportunities Widget</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -935,12 +949,13 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Engagement Health</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>Depends</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -982,12 +997,13 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Activity Feed</t>
+          <t>Activity Feed
+Signals</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1027,12 +1043,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Activity Feed</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1049,7 +1065,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>[C4-Row11] Trigger logic copy not explicitly updated in feedback (only retention given) — left as original.</t>
+          <t>[C4-Row11] Trigger logic copy not explicitly updated in feedback (only retention given) — confirmed correct by stakeholder.</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1092,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Activity Feed</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1123,12 +1139,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Activity Feed</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1168,12 +1184,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Activity Feed</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Data Source</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1240,7 +1256,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>4. 'Where User Can Resolve' is now a single value (Data Source) for every row per latest feedback.</t>
+          <t>4. 'Where User Is Notified' and 'Where User Can Resolve' now vary per row (including N/A and 'Depends') per latest feedback.</t>
         </is>
       </c>
     </row>

</xml_diff>